<commit_message>
Boot to Microsoft Extended BASIC when it is in the ROM
The monitor's reset now copies the ROM to RAM and starts BASIC at $9C00
if the byte there is $7E (JMP), otherwise Assist09 as before. BASIC's
new MONITOR and FLEX commands come back through MONENT via the 6809's
unused reserved vector at $FFF0. $E03C is still the monitor entry used
by FLEX's MON and the clock program.

BASIC itself is Microsoft's code and is not included; docs/basic-port.md
describes the changes to Grant Searle's port, including the bracket
fixes a09 needs for expressions AS9 evaluates left to right.

- monitor: BOOT, MONENT, COPYOFF; reset vector -> BOOT, $FFF0 -> MONENT
- FLEX-core.hex: drop $FF padding at $E884-$E89F, now monitor code
- rom-images: v7 image (without BASIC); v6 kept for reference
- docs: basic-port.md, README, monitor-commands.md/.pdf, added-commands
  spreadsheet, NOTICE.md
- .gitignore: *.lst
</commit_message>
<xml_diff>
--- a/software/docs/Assist09_Added_Commands.xlsx
+++ b/software/docs/Assist09_Added_Commands.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Added commands" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entry points" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -602,6 +603,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Reset</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BOOT (reset vector)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Copies the ROM to RAM, switches the ROM off, masks the RTC interrupt and sets up the console. If BASIC is in the ROM (the byte at $9C00 is $7E, a JMP), it starts BASIC; otherwise it starts Assist09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>$E03C</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Enters Assist09. FLEX's MON command and the clock program's Q jump here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>From BASIC</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>[$FFF0] (MONENT)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rebuilds the monitor's work page, then enters Assist09 if A=0 or boots FLEX (as F does) if A='F'. Used by BASIC's MONITOR and FLEX commands. $FFF0 is the 6809's reserved vector, which the CPU never uses.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -611,7 +699,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>The formatter, loader and clock program sit in ROM above or away from user RAM, so $0000-$BFFF stays free. The clock program at $C000 is restored from the ROM image on every reset.</t>
+          <t>The formatter, loader and clock program sit in ROM above or away from user RAM, so $0000-$BFFF stays free ($0000-$9BFF if BASIC is in the ROM). The clock program at $C000 is restored from the ROM image on every reset.</t>
         </is>
       </c>
     </row>
@@ -632,7 +720,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Image: Monolithic-Flex-Assist09-BIOS-Format-Loader_v6.</t>
+          <t>Image: Monolithic-Flex-Assist09-BIOS-Format-Loader_v7 (without BASIC). Microsoft Extended BASIC can be added at $9C00-$BFEA; it is not included - see basic-port.md.</t>
         </is>
       </c>
     </row>

</xml_diff>